<commit_message>
update: trường Brandname cho các table schema
</commit_message>
<xml_diff>
--- a/public/files/sample_file.xlsx
+++ b/public/files/sample_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\CGV_Telecom_Booking_V1_Front-End\public\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CGV_Telecom_Booking_V1_Front-End\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCD18DCE-33C9-4EE4-AD0A-64E8872A6C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FA21DE-001E-4D17-94DE-188D7CB9D0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F038391C-AC66-43F7-8E29-578F14832AAD}"/>
+    <workbookView xWindow="7035" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{F038391C-AC66-43F7-8E29-578F14832AAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>Số điện thoại</t>
   </si>
@@ -47,18 +47,6 @@
     <t>Loại số</t>
   </si>
   <si>
-    <t>Viettel</t>
-  </si>
-  <si>
-    <t>Số VIP</t>
-  </si>
-  <si>
-    <t>0559517003</t>
-  </si>
-  <si>
-    <t>0328063079</t>
-  </si>
-  <si>
     <t>Phí khởi tạo</t>
   </si>
   <si>
@@ -68,38 +56,47 @@
     <t>Phí số đẹp</t>
   </si>
   <si>
-    <t>0895541178</t>
-  </si>
-  <si>
-    <t>0924552544</t>
-  </si>
-  <si>
-    <t>0982847555</t>
-  </si>
-  <si>
     <t>Chuyển tiếp số</t>
   </si>
   <si>
-    <t>19008898</t>
-  </si>
-  <si>
-    <t>0919098898</t>
-  </si>
-  <si>
     <t>Tên khách hàng</t>
+  </si>
+  <si>
+    <t>Tên brandname</t>
+  </si>
+  <si>
+    <t>0123456789</t>
+  </si>
+  <si>
+    <t>0912345678</t>
+  </si>
+  <si>
+    <t>0887766554</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Brandname 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -124,13 +121,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8126F7F4-9726-480C-98F2-5877011EB363}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.1328125" bestFit="1" customWidth="1"/>
@@ -474,9 +469,10 @@
     <col min="6" max="6" width="15.1328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.6640625" customWidth="1"/>
     <col min="8" max="8" width="16.1328125" customWidth="1"/>
+    <col min="9" max="9" width="15.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -487,143 +483,105 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2000</v>
+      </c>
+      <c r="E2" s="3">
+        <v>3000</v>
+      </c>
+      <c r="F2" s="3">
+        <v>4000</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>16</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2">
+    <row r="3" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3">
         <v>2000</v>
       </c>
-      <c r="E2">
+      <c r="E3" s="3">
         <v>3000</v>
       </c>
-      <c r="F2">
+      <c r="F3" s="3">
         <v>4000</v>
       </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3">
+    <row r="4" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="3">
         <v>2000</v>
       </c>
-      <c r="E3">
+      <c r="E4" s="3">
         <v>3000</v>
       </c>
-      <c r="F3">
+      <c r="F4" s="3">
         <v>4000</v>
       </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4">
-        <v>2000</v>
-      </c>
-      <c r="E4">
-        <v>3000</v>
-      </c>
-      <c r="F4">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>2000</v>
-      </c>
-      <c r="E5">
-        <v>3000</v>
-      </c>
-      <c r="F5">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6">
-        <v>2000</v>
-      </c>
-      <c r="E6">
-        <v>3000</v>
-      </c>
-      <c r="F6">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7">
-        <v>2000</v>
-      </c>
-      <c r="E7">
-        <v>3000</v>
-      </c>
-      <c r="F7">
-        <v>4000</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>15</v>
-      </c>
+    <row r="5" spans="1:9" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>